<commit_message>
feat: revisi nilai tugas GTI skala 60-90 proporsional
- Semua nilai tugas diskalakan ke range 60-90
- Proporsi tetap dijaga (skor tinggi makin tinggi)
- Raw score 37→60, 78→90 (linear scaling)
- 194 mahasiswa, avg 71.7, distribusi merata
- Update semua GTI PAIK/MIK (9 file) + FINAL Excel
</commit_message>
<xml_diff>
--- a/nilai-nilai/gti-2026/GTI_MIK1624406_2025_2_A.xlsx
+++ b/nilai-nilai/gti-2026/GTI_MIK1624406_2025_2_A.xlsx
@@ -34,7 +34,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +56,11 @@
         <fgColor rgb="FFEBF1DE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD7BE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -69,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -85,6 +90,10 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -626,7 +635,7 @@
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="4" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n">
@@ -668,7 +677,7 @@
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="5" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n">
@@ -710,7 +719,7 @@
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="6" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n">
@@ -752,7 +761,7 @@
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="6" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n">
@@ -793,8 +802,8 @@
       </c>
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
-      <c r="G12" s="4" t="n">
-        <v>80</v>
+      <c r="G12" s="6" t="n">
+        <v>84</v>
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n">
@@ -835,8 +844,8 @@
       </c>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n"/>
-      <c r="G13" s="5" t="n">
-        <v>67</v>
+      <c r="G13" s="6" t="n">
+        <v>77</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n">
@@ -878,7 +887,7 @@
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="4" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="n">
@@ -920,7 +929,7 @@
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="4" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n">
@@ -962,7 +971,7 @@
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="6" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="n">
@@ -1003,8 +1012,8 @@
       </c>
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
-      <c r="G17" s="4" t="n">
-        <v>80</v>
+      <c r="G17" s="6" t="n">
+        <v>84</v>
       </c>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n">
@@ -1046,7 +1055,7 @@
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="5" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="3" t="n">
@@ -1088,7 +1097,7 @@
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="6" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="n">
@@ -1130,7 +1139,7 @@
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="5" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n">
@@ -1171,7 +1180,7 @@
       </c>
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
-      <c r="G21" s="5" t="n">
+      <c r="G21" s="7" t="n">
         <v>60</v>
       </c>
       <c r="H21" s="3" t="n"/>
@@ -1214,7 +1223,7 @@
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="5" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n">
@@ -1256,7 +1265,7 @@
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
       <c r="G23" s="5" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n">
@@ -1298,7 +1307,7 @@
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="5" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n">
@@ -1339,8 +1348,8 @@
       </c>
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
-      <c r="G25" s="5" t="n">
-        <v>67</v>
+      <c r="G25" s="6" t="n">
+        <v>77</v>
       </c>
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n">
@@ -1382,7 +1391,7 @@
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n"/>
       <c r="G26" s="6" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n">
@@ -1424,7 +1433,7 @@
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n"/>
       <c r="G27" s="6" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n">
@@ -1466,7 +1475,7 @@
       <c r="E28" s="3" t="n"/>
       <c r="F28" s="3" t="n"/>
       <c r="G28" s="6" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n">
@@ -1508,7 +1517,7 @@
       <c r="E29" s="3" t="n"/>
       <c r="F29" s="3" t="n"/>
       <c r="G29" s="5" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n">
@@ -1550,7 +1559,7 @@
       <c r="E30" s="3" t="n"/>
       <c r="F30" s="3" t="n"/>
       <c r="G30" s="5" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n">
@@ -1592,7 +1601,7 @@
       <c r="E31" s="3" t="n"/>
       <c r="F31" s="3" t="n"/>
       <c r="G31" s="6" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n">
@@ -1633,7 +1642,7 @@
       </c>
       <c r="E32" s="3" t="n"/>
       <c r="F32" s="3" t="n"/>
-      <c r="G32" s="5" t="n">
+      <c r="G32" s="7" t="n">
         <v>60</v>
       </c>
       <c r="H32" s="3" t="n"/>
@@ -1675,8 +1684,8 @@
       </c>
       <c r="E33" s="3" t="n"/>
       <c r="F33" s="3" t="n"/>
-      <c r="G33" s="5" t="n">
-        <v>67</v>
+      <c r="G33" s="6" t="n">
+        <v>77</v>
       </c>
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n">
@@ -1718,7 +1727,7 @@
       <c r="E34" s="3" t="n"/>
       <c r="F34" s="3" t="n"/>
       <c r="G34" s="5" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n">
@@ -1759,7 +1768,7 @@
       </c>
       <c r="E35" s="3" t="n"/>
       <c r="F35" s="3" t="n"/>
-      <c r="G35" s="5" t="n">
+      <c r="G35" s="7" t="n">
         <v>60</v>
       </c>
       <c r="H35" s="3" t="n"/>
@@ -1801,8 +1810,8 @@
       </c>
       <c r="E36" s="3" t="n"/>
       <c r="F36" s="3" t="n"/>
-      <c r="G36" s="5" t="n">
-        <v>67</v>
+      <c r="G36" s="6" t="n">
+        <v>77</v>
       </c>
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n">
@@ -1844,7 +1853,7 @@
       <c r="E37" s="3" t="n"/>
       <c r="F37" s="3" t="n"/>
       <c r="G37" s="5" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n">
@@ -1886,7 +1895,7 @@
       <c r="E38" s="3" t="n"/>
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="5" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n">
@@ -1928,7 +1937,7 @@
       <c r="E39" s="3" t="n"/>
       <c r="F39" s="3" t="n"/>
       <c r="G39" s="5" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n">
@@ -1970,7 +1979,7 @@
       <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="n"/>
       <c r="G40" s="5" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n">
@@ -2012,7 +2021,7 @@
       <c r="E41" s="3" t="n"/>
       <c r="F41" s="3" t="n"/>
       <c r="G41" s="5" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n">
@@ -2054,7 +2063,7 @@
       <c r="E42" s="3" t="n"/>
       <c r="F42" s="3" t="n"/>
       <c r="G42" s="5" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n">
@@ -2096,7 +2105,7 @@
       <c r="E43" s="3" t="n"/>
       <c r="F43" s="3" t="n"/>
       <c r="G43" s="6" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="n">
@@ -2138,7 +2147,7 @@
       <c r="E44" s="3" t="n"/>
       <c r="F44" s="3" t="n"/>
       <c r="G44" s="5" t="n">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="H44" s="3" t="n"/>
       <c r="I44" s="3" t="n">
@@ -2179,7 +2188,7 @@
       </c>
       <c r="E45" s="3" t="n"/>
       <c r="F45" s="3" t="n"/>
-      <c r="G45" s="5" t="n">
+      <c r="G45" s="7" t="n">
         <v>60</v>
       </c>
       <c r="H45" s="3" t="n"/>

</xml_diff>